<commit_message>
correct index.html event trigger
</commit_message>
<xml_diff>
--- a/outputs/Gastos_0529_RJW_2026_jun(1hojas).xlsx
+++ b/outputs/Gastos_0529_RJW_2026_jun(1hojas).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\userRafae\Descargas\martin_gastos\web_app\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0970031-15E3-4730-B887-1BA2D8810900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{583C0B97-B508-41DC-BF30-2D262D8A83EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7E3648A7-F6B8-40B4-8218-6A3BB44BE44D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7EC25613-9AAF-4048-9F07-1D08A2114A4D}"/>
   </bookViews>
   <sheets>
     <sheet name="JUNIO (1)" sheetId="2" r:id="rId1"/>
@@ -1356,7 +1356,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54E7F0CE-91F6-4DF8-91E7-F8BB3BDA0BE6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A95981D3-57CE-439E-ADCA-E96F60D185E9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1727,7 +1727,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD71230-8B2A-4997-A0F5-E98EC5B28587}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D30C98A-D62F-43E0-AC60-03AA58A1D81C}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>